<commit_message>
Handling all envi DB's completed
</commit_message>
<xml_diff>
--- a/DataProvider/db_details.xlsx
+++ b/DataProvider/db_details.xlsx
@@ -9,7 +9,7 @@
   </bookViews>
   <sheets>
     <sheet name="db" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="tables" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="credentials" sheetId="2" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -21,57 +21,57 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="69">
   <si>
     <t xml:space="preserve">DB</t>
   </si>
   <si>
-    <t xml:space="preserve">Demo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demo1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dev1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dev2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dev3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dev4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dev5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dev6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dev7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dev8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dev9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dev10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dev11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dev12</t>
+    <t xml:space="preserve">demo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">demo1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">qa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">perf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dev1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dev2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dev3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dev4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dev5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dev6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dev7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dev8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dev9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dev10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dev11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dev12</t>
   </si>
   <si>
     <t xml:space="preserve">information_schema</t>
@@ -125,10 +125,13 @@
     <t xml:space="preserve">cnpware_demo1</t>
   </si>
   <si>
+    <t xml:space="preserve">config</t>
+  </si>
+  <si>
     <t xml:space="preserve">config_apps</t>
   </si>
   <si>
-    <t xml:space="preserve">config_apps2</t>
+    <t xml:space="preserve">config2</t>
   </si>
   <si>
     <t xml:space="preserve">config_apps_new</t>
@@ -146,6 +149,9 @@
     <t xml:space="preserve">ezetap_demo</t>
   </si>
   <si>
+    <t xml:space="preserve">ezetap_demo1</t>
+  </si>
+  <si>
     <t xml:space="preserve">ezetap_temp</t>
   </si>
   <si>
@@ -204,6 +210,24 @@
   </si>
   <si>
     <t xml:space="preserve">wware</t>
+  </si>
+  <si>
+    <t xml:space="preserve">environment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">username</t>
+  </si>
+  <si>
+    <t xml:space="preserve">password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ezedemo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">abc123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ezedemo1</t>
   </si>
 </sst>
 </file>
@@ -213,11 +237,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -239,12 +264,21 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="JetBrains Mono"/>
       <family val="3"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -302,7 +336,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -316,6 +350,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -397,12 +435,15 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q33"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="25.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="20.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="11" style="0" width="18.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="20.45"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -468,18 +509,30 @@
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
+      <c r="F2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="H2" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
+      <c r="K2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="N2" s="2"/>
-      <c r="O2" s="2"/>
+      <c r="O2" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="P2" s="3" t="s">
         <v>17</v>
       </c>
@@ -495,18 +548,30 @@
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="F3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="H3" s="2" t="s">
         <v>19</v>
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
+      <c r="K3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
+      <c r="O3" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="P3" s="2" t="s">
         <v>19</v>
       </c>
@@ -522,18 +587,30 @@
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
+      <c r="F4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>20</v>
+      </c>
       <c r="H4" s="2" t="s">
         <v>20</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
+      <c r="K4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>20</v>
+      </c>
       <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
+      <c r="O4" s="2" t="s">
+        <v>20</v>
+      </c>
       <c r="P4" s="2" t="s">
         <v>21</v>
       </c>
@@ -555,7 +632,9 @@
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
+      <c r="L5" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
@@ -641,7 +720,9 @@
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
+      <c r="F9" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2" t="s">
         <v>27</v>
@@ -650,7 +731,9 @@
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
+      <c r="M9" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
       <c r="P9" s="2" t="s">
@@ -668,25 +751,37 @@
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
+      <c r="F10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="H10" s="2" t="s">
         <v>30</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
+      <c r="K10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="N10" s="2"/>
-      <c r="O10" s="2"/>
+      <c r="O10" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="P10" s="2" t="s">
         <v>31</v>
       </c>
       <c r="Q10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="4" t="s">
         <v>32</v>
       </c>
       <c r="B11" s="2"/>
@@ -701,7 +796,9 @@
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
+      <c r="L11" s="2" t="s">
+        <v>31</v>
+      </c>
       <c r="M11" s="2"/>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
@@ -709,193 +806,277 @@
       <c r="Q11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="4" t="s">
         <v>34</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
+      <c r="F12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>35</v>
+      </c>
       <c r="H12" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
-      <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
+      <c r="K12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="M12" s="2" t="s">
+        <v>35</v>
+      </c>
       <c r="N12" s="2"/>
-      <c r="O12" s="2"/>
+      <c r="O12" s="2" t="s">
+        <v>35</v>
+      </c>
       <c r="P12" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
-        <v>35</v>
+      <c r="A13" s="4" t="s">
+        <v>36</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
+      <c r="F13" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>37</v>
+      </c>
       <c r="H13" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
+      <c r="K13" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>37</v>
+      </c>
       <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
+      <c r="O13" s="2" t="s">
+        <v>37</v>
+      </c>
       <c r="P13" s="2"/>
       <c r="Q13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
-        <v>37</v>
+      <c r="A14" s="4" t="s">
+        <v>38</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
+      <c r="F14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>38</v>
+      </c>
       <c r="H14" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
+      <c r="K14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>38</v>
+      </c>
       <c r="N14" s="2"/>
-      <c r="O14" s="2"/>
+      <c r="O14" s="2" t="s">
+        <v>38</v>
+      </c>
       <c r="P14" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Q14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
+      <c r="F15" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="H15" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
+      <c r="K15" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="N15" s="2"/>
-      <c r="O15" s="2"/>
+      <c r="O15" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="P15" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="Q15" s="2"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
+      <c r="F16" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>40</v>
+      </c>
       <c r="H16" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
-      <c r="M16" s="2"/>
+      <c r="K16" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>40</v>
+      </c>
       <c r="N16" s="2"/>
-      <c r="O16" s="2"/>
+      <c r="O16" s="2" t="s">
+        <v>40</v>
+      </c>
       <c r="P16" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="Q16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
+      <c r="F17" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>41</v>
+      </c>
       <c r="H17" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2"/>
+      <c r="K17" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>41</v>
+      </c>
       <c r="N17" s="2"/>
-      <c r="O17" s="2"/>
+      <c r="O17" s="2" t="s">
+        <v>41</v>
+      </c>
       <c r="P17" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
+      <c r="F18" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="H18" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
-      <c r="L18" s="2"/>
-      <c r="M18" s="2"/>
+      <c r="K18" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="N18" s="2"/>
-      <c r="O18" s="2"/>
+      <c r="O18" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="P18" s="2"/>
       <c r="Q18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -904,7 +1085,7 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
@@ -918,45 +1099,49 @@
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
+      <c r="K20" s="2" t="s">
+        <v>45</v>
+      </c>
       <c r="L20" s="2"/>
-      <c r="M20" s="2"/>
+      <c r="M20" s="2" t="s">
+        <v>45</v>
+      </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
       <c r="P20" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="Q20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
@@ -966,69 +1151,93 @@
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
       <c r="P21" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="Q21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
+      <c r="F22" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="H22" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
-      <c r="L22" s="2"/>
-      <c r="M22" s="2"/>
+      <c r="K22" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="M22" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="N22" s="2"/>
-      <c r="O22" s="2"/>
+      <c r="O22" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="P22" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Q22" s="2"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
+      <c r="F23" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="H23" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
-      <c r="L23" s="2"/>
-      <c r="M23" s="2"/>
+      <c r="K23" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="L23" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="M23" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="N23" s="2"/>
-      <c r="O23" s="2"/>
+      <c r="O23" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="P23" s="2"/>
       <c r="Q23" s="2"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
@@ -1047,65 +1256,89 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
+      <c r="F25" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>53</v>
+      </c>
       <c r="H25" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
-      <c r="L25" s="2"/>
-      <c r="M25" s="2"/>
+      <c r="K25" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="L25" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="M25" s="2" t="s">
+        <v>53</v>
+      </c>
       <c r="N25" s="2"/>
-      <c r="O25" s="2"/>
+      <c r="O25" s="2" t="s">
+        <v>53</v>
+      </c>
       <c r="P25" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="Q25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
+      <c r="F26" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>55</v>
+      </c>
       <c r="H26" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
-      <c r="K26" s="2"/>
-      <c r="L26" s="2"/>
-      <c r="M26" s="2"/>
+      <c r="K26" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="L26" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="M26" s="2" t="s">
+        <v>55</v>
+      </c>
       <c r="N26" s="2"/>
-      <c r="O26" s="2"/>
+      <c r="O26" s="2" t="s">
+        <v>55</v>
+      </c>
       <c r="P26" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="Q26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
@@ -1124,11 +1357,11 @@
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
@@ -1147,11 +1380,11 @@
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B29" s="2"/>
       <c r="C29" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
@@ -1170,11 +1403,11 @@
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
@@ -1193,38 +1426,50 @@
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B31" s="2"/>
       <c r="C31" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
+      <c r="F31" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="H31" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
-      <c r="K31" s="2"/>
-      <c r="L31" s="2"/>
-      <c r="M31" s="2"/>
+      <c r="K31" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="L31" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="M31" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="N31" s="2"/>
-      <c r="O31" s="2"/>
+      <c r="O31" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="P31" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="Q31" s="2"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B32" s="2"/>
       <c r="C32" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
@@ -1243,28 +1488,40 @@
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B33" s="2"/>
       <c r="C33" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
+      <c r="F33" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>62</v>
+      </c>
       <c r="H33" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
-      <c r="K33" s="2"/>
-      <c r="L33" s="2"/>
-      <c r="M33" s="2"/>
+      <c r="K33" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="L33" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M33" s="2" t="s">
+        <v>62</v>
+      </c>
       <c r="N33" s="2"/>
-      <c r="O33" s="2"/>
+      <c r="O33" s="2" t="s">
+        <v>62</v>
+      </c>
       <c r="P33" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q33" s="2"/>
     </row>
@@ -1284,12 +1541,204 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10.89"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>

</xml_diff>

<commit_message>
update message in the test case.
</commit_message>
<xml_diff>
--- a/DataProvider/db_details.xlsx
+++ b/DataProvider/db_details.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="db" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="70">
   <si>
     <t xml:space="preserve">DB</t>
   </si>
@@ -72,6 +72,9 @@
   </si>
   <si>
     <t xml:space="preserve">dev12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dev16</t>
   </si>
   <si>
     <t xml:space="preserve">information_schema</t>
@@ -434,18 +437,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q33"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:R33"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="25.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18.77"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="18.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="11" style="0" width="18.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="10" style="0" width="18.77"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="20.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="18.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="17" style="0" width="18.77"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -500,143 +502,155 @@
       <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N2" s="2"/>
       <c r="O2" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="N3" s="2"/>
       <c r="O3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N4" s="2"/>
       <c r="O4" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="Q4" s="2" t="s">
-        <v>20</v>
+      <c r="R4" s="2" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
@@ -647,21 +661,22 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -677,14 +692,15 @@
       <c r="O6" s="2"/>
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
+      <c r="R6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
@@ -700,14 +716,15 @@
       <c r="O7" s="2"/>
       <c r="P7" s="2"/>
       <c r="Q7" s="2"/>
+      <c r="R7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
@@ -723,90 +740,97 @@
       <c r="O8" s="2"/>
       <c r="P8" s="2"/>
       <c r="Q8" s="2"/>
+      <c r="R8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
       <c r="M9" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
       <c r="P9" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="R9" s="2" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="Q10" s="2" t="s">
-        <v>30</v>
+      <c r="R10" s="2" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
@@ -817,314 +841,336 @@
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M11" s="2"/>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
       <c r="P11" s="2"/>
       <c r="Q11" s="2"/>
+      <c r="R11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P12" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
+      </c>
+      <c r="R12" s="2" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I13" s="2"/>
       <c r="J13" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N13" s="2"/>
       <c r="O13" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P13" s="2"/>
       <c r="Q13" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
+      </c>
+      <c r="R13" s="2" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="Q14" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="R14" s="2" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I15" s="2"/>
       <c r="J15" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P15" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="Q15" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
+      </c>
+      <c r="R15" s="2" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P16" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q16" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
+      </c>
+      <c r="R16" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I17" s="2"/>
       <c r="J17" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="P17" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q17" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
+      </c>
+      <c r="R17" s="2" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="I18" s="2"/>
       <c r="J18" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="P18" s="2"/>
       <c r="Q18" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
+      </c>
+      <c r="R18" s="2" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -1133,7 +1179,7 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
@@ -1144,54 +1190,58 @@
       <c r="O19" s="2"/>
       <c r="P19" s="2"/>
       <c r="Q19" s="2"/>
+      <c r="R19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="L20" s="2"/>
       <c r="M20" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
       <c r="P20" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q20" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
+      </c>
+      <c r="R20" s="2" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
@@ -1201,103 +1251,112 @@
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
       <c r="P21" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="Q21" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
+      </c>
+      <c r="R21" s="2" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I22" s="2"/>
       <c r="J22" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="P22" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q22" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
+      </c>
+      <c r="R22" s="2" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I23" s="2"/>
       <c r="J23" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="N23" s="2"/>
       <c r="O23" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="P23" s="2"/>
       <c r="Q23" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
+      </c>
+      <c r="R23" s="2" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
@@ -1313,100 +1372,107 @@
       <c r="O24" s="2"/>
       <c r="P24" s="2"/>
       <c r="Q24" s="2"/>
+      <c r="R24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
       <c r="F25" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I25" s="2"/>
       <c r="J25" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L25" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="P25" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="Q25" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
+      </c>
+      <c r="R25" s="2" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
       <c r="F26" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I26" s="2"/>
       <c r="J26" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N26" s="2"/>
       <c r="O26" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="P26" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Q26" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
+      </c>
+      <c r="R26" s="2" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
@@ -1422,14 +1488,15 @@
       <c r="O27" s="2"/>
       <c r="P27" s="2"/>
       <c r="Q27" s="2"/>
+      <c r="R27" s="2"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
@@ -1445,14 +1512,15 @@
       <c r="O28" s="2"/>
       <c r="P28" s="2"/>
       <c r="Q28" s="2"/>
+      <c r="R28" s="2"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B29" s="2"/>
       <c r="C29" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
@@ -1468,14 +1536,15 @@
       <c r="O29" s="2"/>
       <c r="P29" s="2"/>
       <c r="Q29" s="2"/>
+      <c r="R29" s="2"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
@@ -1491,57 +1560,61 @@
       <c r="O30" s="2"/>
       <c r="P30" s="2"/>
       <c r="Q30" s="2"/>
+      <c r="R30" s="2"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B31" s="2"/>
       <c r="C31" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
       <c r="F31" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I31" s="2"/>
       <c r="J31" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="P31" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="Q31" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
+      </c>
+      <c r="R31" s="2" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B32" s="2"/>
       <c r="C32" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
@@ -1557,54 +1630,58 @@
       <c r="O32" s="2"/>
       <c r="P32" s="2"/>
       <c r="Q32" s="2"/>
+      <c r="R32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B33" s="2"/>
       <c r="C33" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
       <c r="F33" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I33" s="2"/>
       <c r="J33" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="P33" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q33" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
+      </c>
+      <c r="R33" s="2" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
@@ -1617,8 +1694,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10.89"/>
@@ -1626,13 +1703,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1640,10 +1717,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1651,10 +1728,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1662,10 +1739,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1673,10 +1750,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1684,10 +1761,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1695,10 +1772,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1706,10 +1783,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1717,10 +1794,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1728,10 +1805,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1739,10 +1816,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1750,10 +1827,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1761,10 +1838,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1772,10 +1849,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1783,10 +1860,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1794,10 +1871,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1805,16 +1882,27 @@
         <v>16</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C17" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="s">
         <v>67</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>

</xml_diff>

<commit_message>
updated ezewallet variable names
</commit_message>
<xml_diff>
--- a/DataProvider/db_details.xlsx
+++ b/DataProvider/db_details.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="db" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="70">
   <si>
     <t xml:space="preserve">DB</t>
   </si>
@@ -134,10 +134,10 @@
     <t xml:space="preserve">config_apps</t>
   </si>
   <si>
+    <t xml:space="preserve">config_apps_new</t>
+  </si>
+  <si>
     <t xml:space="preserve">config2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">config_apps_new</t>
   </si>
   <si>
     <t xml:space="preserve">ea</t>
@@ -438,7 +438,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:R33"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="25.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25.4"/>
@@ -447,7 +447,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18.77"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="10" style="0" width="18.77"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="20.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="17" style="0" width="18.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="18.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="20.45"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -548,7 +549,7 @@
       <c r="Q2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="R2" s="3" t="s">
         <v>18</v>
       </c>
     </row>
@@ -641,7 +642,7 @@
         <v>21</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -893,52 +894,50 @@
         <v>36</v>
       </c>
       <c r="R12" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I13" s="2"/>
       <c r="J13" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="N13" s="2"/>
       <c r="O13" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P13" s="2"/>
       <c r="Q13" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="R13" s="2" t="s">
-        <v>38</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="R13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
@@ -1164,9 +1163,7 @@
       <c r="Q18" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="R18" s="2" t="s">
-        <v>44</v>
-      </c>
+      <c r="R18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
@@ -1346,9 +1343,7 @@
       <c r="Q23" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="R23" s="2" t="s">
-        <v>52</v>
-      </c>
+      <c r="R23" s="2"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
@@ -1681,7 +1676,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
@@ -1695,7 +1690,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C18"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10.89"/>
@@ -1892,7 +1887,7 @@
       <c r="A18" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="4" t="s">
         <v>67</v>
       </c>
       <c r="C18" s="2" t="s">
@@ -1902,7 +1897,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>

</xml_diff>

<commit_message>
EzeGro test cases Added
</commit_message>
<xml_diff>
--- a/DataProvider/db_details.xlsx
+++ b/DataProvider/db_details.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="74">
   <si>
     <t xml:space="preserve">DB</t>
   </si>
@@ -77,6 +77,9 @@
     <t xml:space="preserve">dev16</t>
   </si>
   <si>
+    <t xml:space="preserve">qa-rc</t>
+  </si>
+  <si>
     <t xml:space="preserve">information_schema</t>
   </si>
   <si>
@@ -219,6 +222,9 @@
   </si>
   <si>
     <t xml:space="preserve">instant_settlement_details</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ezestore</t>
   </si>
   <si>
     <t xml:space="preserve">environment</t>
@@ -447,8 +453,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R34"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:S35"/>
+  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="25.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25.4"/>
@@ -458,7 +464,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="10" style="0" width="18.77"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="20.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="18.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="20.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="18" style="0" width="20.45"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -516,152 +522,164 @@
       <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="N2" s="2"/>
       <c r="O2" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N3" s="2"/>
       <c r="O3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="N4" s="2"/>
       <c r="O4" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="Q4" s="2" t="s">
-        <v>21</v>
-      </c>
       <c r="R4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="S4" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
@@ -672,7 +690,7 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
@@ -680,14 +698,15 @@
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
       <c r="R5" s="2"/>
+      <c r="S5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -704,14 +723,15 @@
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
       <c r="R6" s="2"/>
+      <c r="S6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
@@ -728,14 +748,15 @@
       <c r="P7" s="2"/>
       <c r="Q7" s="2"/>
       <c r="R7" s="2"/>
+      <c r="S7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
@@ -752,96 +773,103 @@
       <c r="P8" s="2"/>
       <c r="Q8" s="2"/>
       <c r="R8" s="2"/>
+      <c r="S8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
       <c r="M9" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
       <c r="P9" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="S9" s="2" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P10" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q10" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="Q10" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="R10" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="S10" s="2" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
@@ -852,7 +880,7 @@
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="M11" s="2"/>
       <c r="N11" s="2"/>
@@ -860,324 +888,342 @@
       <c r="P11" s="2"/>
       <c r="Q11" s="2"/>
       <c r="R11" s="2"/>
+      <c r="S11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="P12" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R12" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
+      </c>
+      <c r="S12" s="2" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I13" s="2"/>
       <c r="J13" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N13" s="2"/>
       <c r="O13" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P13" s="2"/>
       <c r="Q13" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="R13" s="2"/>
+      <c r="S13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="Q14" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="R14" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
+      </c>
+      <c r="S14" s="2" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I15" s="2"/>
       <c r="J15" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P15" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q15" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="R15" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
+      </c>
+      <c r="S15" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="P16" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q16" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="R16" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
+      </c>
+      <c r="S16" s="2" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I17" s="2"/>
       <c r="J17" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="P17" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q17" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="R17" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
+      </c>
+      <c r="S17" s="2" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I18" s="2"/>
       <c r="J18" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="P18" s="2"/>
       <c r="Q18" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="R18" s="2"/>
+      <c r="S18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -1186,7 +1232,7 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
@@ -1198,57 +1244,61 @@
       <c r="P19" s="2"/>
       <c r="Q19" s="2"/>
       <c r="R19" s="2"/>
+      <c r="S19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="L20" s="2"/>
       <c r="M20" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
       <c r="P20" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="Q20" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="R20" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
+      </c>
+      <c r="S20" s="2" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
@@ -1258,110 +1308,117 @@
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
       <c r="P21" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q21" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="R21" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
+      </c>
+      <c r="S21" s="2" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I22" s="2"/>
       <c r="J22" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="P22" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q22" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="R22" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
+      </c>
+      <c r="S22" s="2" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I23" s="2"/>
       <c r="J23" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N23" s="2"/>
       <c r="O23" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="P23" s="2"/>
       <c r="Q23" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="R23" s="2"/>
+      <c r="S23" s="2"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
@@ -1378,106 +1435,113 @@
       <c r="P24" s="2"/>
       <c r="Q24" s="2"/>
       <c r="R24" s="2"/>
+      <c r="S24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
       <c r="F25" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I25" s="2"/>
       <c r="J25" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="L25" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="P25" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Q25" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="R25" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
+      </c>
+      <c r="S25" s="2" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
       <c r="F26" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I26" s="2"/>
       <c r="J26" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N26" s="2"/>
       <c r="O26" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="P26" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q26" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="R26" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
+      </c>
+      <c r="S26" s="2" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
@@ -1494,14 +1558,15 @@
       <c r="P27" s="2"/>
       <c r="Q27" s="2"/>
       <c r="R27" s="2"/>
+      <c r="S27" s="2"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
@@ -1518,14 +1583,15 @@
       <c r="P28" s="2"/>
       <c r="Q28" s="2"/>
       <c r="R28" s="2"/>
+      <c r="S28" s="2"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B29" s="2"/>
       <c r="C29" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
@@ -1542,14 +1608,15 @@
       <c r="P29" s="2"/>
       <c r="Q29" s="2"/>
       <c r="R29" s="2"/>
+      <c r="S29" s="2"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
@@ -1566,60 +1633,64 @@
       <c r="P30" s="2"/>
       <c r="Q30" s="2"/>
       <c r="R30" s="2"/>
+      <c r="S30" s="2"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B31" s="2"/>
       <c r="C31" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
       <c r="F31" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I31" s="2"/>
       <c r="J31" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="P31" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Q31" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="R31" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
+      </c>
+      <c r="S31" s="2" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B32" s="2"/>
       <c r="C32" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
@@ -1636,56 +1707,60 @@
       <c r="P32" s="2"/>
       <c r="Q32" s="2"/>
       <c r="R32" s="2"/>
+      <c r="S32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B33" s="2"/>
       <c r="C33" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
       <c r="F33" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I33" s="2"/>
       <c r="J33" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="P33" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q33" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="R33" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
+      </c>
+      <c r="S33" s="2" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B34" s="5"/>
       <c r="C34" s="2"/>
@@ -1693,7 +1768,7 @@
       <c r="E34" s="5"/>
       <c r="F34" s="2"/>
       <c r="G34" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H34" s="2"/>
       <c r="I34" s="5"/>
@@ -1706,6 +1781,32 @@
       <c r="P34" s="2"/>
       <c r="Q34" s="2"/>
       <c r="R34" s="2"/>
+      <c r="S34" s="2"/>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B35" s="5"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
+      <c r="I35" s="5"/>
+      <c r="J35" s="2"/>
+      <c r="K35" s="2"/>
+      <c r="L35" s="2"/>
+      <c r="M35" s="2"/>
+      <c r="N35" s="2"/>
+      <c r="O35" s="2"/>
+      <c r="P35" s="2"/>
+      <c r="Q35" s="2"/>
+      <c r="R35" s="2"/>
+      <c r="S35" s="5" t="s">
+        <v>67</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1723,8 +1824,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:C19"/>
+  <sheetFormatPr defaultColWidth="11.66796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10.89"/>
@@ -1732,13 +1833,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1746,10 +1847,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1757,10 +1858,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1768,10 +1869,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1779,10 +1880,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1790,10 +1891,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1801,10 +1902,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1812,10 +1913,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1823,10 +1924,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1834,10 +1935,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1845,10 +1946,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1856,10 +1957,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1867,10 +1968,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1878,10 +1979,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1889,10 +1990,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1900,10 +2001,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1911,10 +2012,10 @@
         <v>16</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1922,10 +2023,21 @@
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Development of merchant portal automation and updated 10 test cases using playwright.
</commit_message>
<xml_diff>
--- a/DataProvider/db_details.xlsx
+++ b/DataProvider/db_details.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="db" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="75">
   <si>
     <t xml:space="preserve">DB</t>
   </si>
@@ -78,6 +78,9 @@
   </si>
   <si>
     <t xml:space="preserve">qa-rc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dev17</t>
   </si>
   <si>
     <t xml:space="preserve">information_schema</t>
@@ -453,8 +456,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:S35"/>
-  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:T35"/>
+  <sheetFormatPr defaultColWidth="11.7421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="25.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25.4"/>
@@ -464,7 +467,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="10" style="0" width="18.77"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="20.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="18.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="18" style="0" width="20.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="18" style="0" width="20.45"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -525,161 +528,173 @@
       <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="N2" s="2"/>
       <c r="O2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="N3" s="2"/>
       <c r="O3" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="N4" s="2"/>
       <c r="O4" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="Q4" s="2" t="s">
-        <v>22</v>
-      </c>
       <c r="R4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="S4" s="2" t="s">
-        <v>22</v>
+      <c r="T4" s="2" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
@@ -690,7 +705,7 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
@@ -699,14 +714,15 @@
       <c r="Q5" s="2"/>
       <c r="R5" s="2"/>
       <c r="S5" s="2"/>
+      <c r="T5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -724,14 +740,15 @@
       <c r="Q6" s="2"/>
       <c r="R6" s="2"/>
       <c r="S6" s="2"/>
+      <c r="T6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
@@ -749,14 +766,15 @@
       <c r="Q7" s="2"/>
       <c r="R7" s="2"/>
       <c r="S7" s="2"/>
+      <c r="T7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
@@ -774,102 +792,109 @@
       <c r="Q8" s="2"/>
       <c r="R8" s="2"/>
       <c r="S8" s="2"/>
+      <c r="T8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
       <c r="M9" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
       <c r="P9" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="S9" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="T9" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q10" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="Q10" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="R10" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S10" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="T10" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
@@ -880,7 +905,7 @@
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="M11" s="2"/>
       <c r="N11" s="2"/>
@@ -889,341 +914,359 @@
       <c r="Q11" s="2"/>
       <c r="R11" s="2"/>
       <c r="S11" s="2"/>
+      <c r="T11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P12" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="R12" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="S12" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="T12" s="2" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I13" s="2"/>
       <c r="J13" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="N13" s="2"/>
       <c r="O13" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P13" s="2"/>
       <c r="Q13" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="R13" s="2"/>
       <c r="S13" s="2"/>
+      <c r="T13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q14" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="R14" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="S14" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
+      </c>
+      <c r="T14" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I15" s="2"/>
       <c r="J15" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="P15" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q15" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="R15" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="S15" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
+      </c>
+      <c r="T15" s="2" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="P16" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q16" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="R16" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="S16" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
+      </c>
+      <c r="T16" s="2" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="I17" s="2"/>
       <c r="J17" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="P17" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q17" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="R17" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="S17" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
+      </c>
+      <c r="T17" s="2" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I18" s="2"/>
       <c r="J18" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="P18" s="2"/>
       <c r="Q18" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="R18" s="2"/>
       <c r="S18" s="2"/>
+      <c r="T18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -1232,7 +1275,7 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
@@ -1245,60 +1288,64 @@
       <c r="Q19" s="2"/>
       <c r="R19" s="2"/>
       <c r="S19" s="2"/>
+      <c r="T19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="L20" s="2"/>
       <c r="M20" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
       <c r="P20" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q20" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="R20" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S20" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
+      </c>
+      <c r="T20" s="2" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
@@ -1308,117 +1355,124 @@
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
       <c r="P21" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q21" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="R21" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="S21" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
+      </c>
+      <c r="T21" s="2" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I22" s="2"/>
       <c r="J22" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="P22" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q22" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="R22" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S22" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
+      </c>
+      <c r="T22" s="2" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I23" s="2"/>
       <c r="J23" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="N23" s="2"/>
       <c r="O23" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="P23" s="2"/>
       <c r="Q23" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R23" s="2"/>
       <c r="S23" s="2"/>
+      <c r="T23" s="2"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
@@ -1436,112 +1490,119 @@
       <c r="Q24" s="2"/>
       <c r="R24" s="2"/>
       <c r="S24" s="2"/>
+      <c r="T24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
       <c r="F25" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I25" s="2"/>
       <c r="J25" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L25" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="P25" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Q25" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="R25" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="S25" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
+      </c>
+      <c r="T25" s="2" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
       <c r="F26" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="I26" s="2"/>
       <c r="J26" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N26" s="2"/>
       <c r="O26" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P26" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q26" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="R26" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="S26" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
+      </c>
+      <c r="T26" s="2" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
@@ -1559,14 +1620,15 @@
       <c r="Q27" s="2"/>
       <c r="R27" s="2"/>
       <c r="S27" s="2"/>
+      <c r="T27" s="2"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
@@ -1584,14 +1646,15 @@
       <c r="Q28" s="2"/>
       <c r="R28" s="2"/>
       <c r="S28" s="2"/>
+      <c r="T28" s="2"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B29" s="2"/>
       <c r="C29" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
@@ -1609,14 +1672,15 @@
       <c r="Q29" s="2"/>
       <c r="R29" s="2"/>
       <c r="S29" s="2"/>
+      <c r="T29" s="2"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
@@ -1634,63 +1698,67 @@
       <c r="Q30" s="2"/>
       <c r="R30" s="2"/>
       <c r="S30" s="2"/>
+      <c r="T30" s="2"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B31" s="2"/>
       <c r="C31" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
       <c r="F31" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I31" s="2"/>
       <c r="J31" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="P31" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q31" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="R31" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S31" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
+      </c>
+      <c r="T31" s="2" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B32" s="2"/>
       <c r="C32" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
@@ -1708,59 +1776,63 @@
       <c r="Q32" s="2"/>
       <c r="R32" s="2"/>
       <c r="S32" s="2"/>
+      <c r="T32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B33" s="2"/>
       <c r="C33" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
       <c r="F33" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I33" s="2"/>
       <c r="J33" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="P33" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="Q33" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="R33" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="S33" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
+      </c>
+      <c r="T33" s="2" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B34" s="5"/>
       <c r="C34" s="2"/>
@@ -1768,7 +1840,7 @@
       <c r="E34" s="5"/>
       <c r="F34" s="2"/>
       <c r="G34" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H34" s="2"/>
       <c r="I34" s="5"/>
@@ -1782,10 +1854,11 @@
       <c r="Q34" s="2"/>
       <c r="R34" s="2"/>
       <c r="S34" s="2"/>
+      <c r="T34" s="2"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B35" s="5"/>
       <c r="C35" s="2"/>
@@ -1805,13 +1878,14 @@
       <c r="Q35" s="2"/>
       <c r="R35" s="2"/>
       <c r="S35" s="5" t="s">
-        <v>67</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="T35" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
@@ -1824,8 +1898,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
-  <sheetFormatPr defaultColWidth="11.66796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10.89"/>
@@ -1833,13 +1907,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1847,10 +1921,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1858,10 +1932,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1869,10 +1943,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1880,10 +1954,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1891,10 +1965,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1902,10 +1976,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1913,10 +1987,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1924,10 +1998,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1935,10 +2009,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1946,10 +2020,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1957,10 +2031,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1968,10 +2042,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1979,10 +2053,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1990,10 +2064,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2001,10 +2075,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2012,10 +2086,10 @@
         <v>16</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2023,10 +2097,10 @@
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2034,16 +2108,27 @@
         <v>18</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C19" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>72</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>

</xml_diff>